<commit_message>
finished BOM and added resources and started layout
</commit_message>
<xml_diff>
--- a/RESOURCES/BOM/BOM.xlsx
+++ b/RESOURCES/BOM/BOM.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://steelwaybuildingsystems-my.sharepoint.com/personal/travis_maginnis_steelway_com/Documents/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nicoj\Documents\Repositories\MIST\RESOURCES\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{57379FDE-D78F-4086-8D61-D2AC360E9294}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3385EE7-1C50-47BB-936D-302565A7D705}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{26158271-47B5-455E-A3AA-B8B46F5ACF1D}"/>
+    <workbookView xWindow="2280" yWindow="2280" windowWidth="19200" windowHeight="11170" xr2:uid="{26158271-47B5-455E-A3AA-B8B46F5ACF1D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="88">
   <si>
     <t xml:space="preserve">Bill Of Material - Project Template </t>
   </si>
@@ -110,12 +110,6 @@
     <t>R6, R7</t>
   </si>
   <si>
-    <t>TH1</t>
-  </si>
-  <si>
-    <t>D1</t>
-  </si>
-  <si>
     <t>J2</t>
   </si>
   <si>
@@ -125,12 +119,6 @@
     <t>USB Type C Power Only</t>
   </si>
   <si>
-    <t>RGB LED</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10K Thermoistor </t>
-  </si>
-  <si>
     <t>10k Resistor</t>
   </si>
   <si>
@@ -143,97 +131,175 @@
     <t>C5</t>
   </si>
   <si>
+    <t>0805 (2012 Metric)</t>
+  </si>
+  <si>
+    <t>KEMET</t>
+  </si>
+  <si>
+    <t>100nF Ceramic Capacitor</t>
+  </si>
+  <si>
+    <t>22pF Ceramic Capacitor</t>
+  </si>
+  <si>
+    <t>22uF Ceramic Capacitor</t>
+  </si>
+  <si>
+    <t>1206 (3216 Metric)</t>
+  </si>
+  <si>
+    <t>https://www.digikey.ca/en/products/detail/same-sky-formerly-cui-devices/UJC-H-G-SMT-P6-TR/24818614</t>
+  </si>
+  <si>
+    <t>Tactile Switch</t>
+  </si>
+  <si>
+    <t>4-SMD (3.2x2.5)</t>
+  </si>
+  <si>
+    <t>https://www.digikey.ca/en/products/detail/abracon-llc/ABM8-16.000MHZ-B2X-T/12349981</t>
+  </si>
+  <si>
+    <t>https://www.digikey.ca/en/products/detail/murata-electronics/GRM21A5C2D220JW01D/6606256</t>
+  </si>
+  <si>
+    <t>https://www.digikey.ca/en/products/detail/murata-electronics/GRM21BZ70J226ME44K/19560602</t>
+  </si>
+  <si>
+    <t>https://www.digikey.ca/en/products/detail/kemet/C0805C104J5RACAUTO/3314435</t>
+  </si>
+  <si>
+    <t>https://www.digikey.ca/en/products/detail/w-rth-elektronik/560112132015/24849722</t>
+  </si>
+  <si>
+    <t>https://www.digikey.ca/en/products/detail/bourns-inc/CRM1206AJW-103ELF/8258196</t>
+  </si>
+  <si>
+    <t>https://www.digikey.ca/en/products/detail/bourns-inc/CR1206-JW-512ELF/3925471</t>
+  </si>
+  <si>
+    <t>https://www.digikey.ca/en/products/detail/alps-alpine/SKRPABE010/18768948</t>
+  </si>
+  <si>
+    <t>Total:</t>
+  </si>
+  <si>
+    <t>Littlefuse</t>
+  </si>
+  <si>
+    <t>Bourns</t>
+  </si>
+  <si>
+    <t>Würth Elektronik</t>
+  </si>
+  <si>
+    <t>Murata Electronics</t>
+  </si>
+  <si>
+    <t>Abracon LLC</t>
+  </si>
+  <si>
+    <t>Same Sky</t>
+  </si>
+  <si>
+    <t>Alpine</t>
+  </si>
+  <si>
+    <t>Analog Devices Inc./Maxim Integrated</t>
+  </si>
+  <si>
+    <t>LED Driver 24-SOIC</t>
+  </si>
+  <si>
+    <t>U2</t>
+  </si>
+  <si>
+    <t>24-SOIC (0.295", 7.50mm Width)</t>
+  </si>
+  <si>
+    <t>https://www.digikey.ca/en/products/detail/analog-devices-inc-maxim-integrated/MAX7219CWG-T/1514450</t>
+  </si>
+  <si>
+    <t>On Hand</t>
+  </si>
+  <si>
+    <t>8x8 LED Matrix</t>
+  </si>
+  <si>
     <t>THT</t>
   </si>
   <si>
-    <t>5MM LED</t>
-  </si>
-  <si>
-    <t>0805 (2012 Metric)</t>
-  </si>
-  <si>
-    <t>KEMET</t>
-  </si>
-  <si>
-    <t>100nF Ceramic Capacitor</t>
-  </si>
-  <si>
-    <t>22pF Ceramic Capacitor</t>
-  </si>
-  <si>
-    <t>22uF Ceramic Capacitor</t>
-  </si>
-  <si>
-    <t>1206 (3216 Metric)</t>
-  </si>
-  <si>
-    <t>https://www.digikey.ca/en/products/detail/same-sky-formerly-cui-devices/UJC-H-G-SMT-P6-TR/24818614</t>
-  </si>
-  <si>
-    <t>Tactile Switch</t>
-  </si>
-  <si>
-    <t>4-SMD (3.2x2.5)</t>
-  </si>
-  <si>
-    <t>https://www.digikey.ca/en/products/detail/abracon-llc/ABM8-16.000MHZ-B2X-T/12349981</t>
-  </si>
-  <si>
-    <t>https://www.digikey.ca/en/products/detail/murata-electronics/GRM21A5C2D220JW01D/6606256</t>
-  </si>
-  <si>
-    <t>https://www.digikey.ca/en/products/detail/murata-electronics/GRM21BZ70J226ME44K/19560602</t>
-  </si>
-  <si>
-    <t>https://www.digikey.ca/en/products/detail/kemet/C0805C104J5RACAUTO/3314435</t>
-  </si>
-  <si>
-    <t>https://www.digikey.ca/en/products/detail/w-rth-elektronik/560112132015/24849722</t>
-  </si>
-  <si>
-    <t>https://www.digikey.ca/en/products/detail/bourns-inc/CRM1206AJW-103ELF/8258196</t>
-  </si>
-  <si>
-    <t>https://www.digikey.ca/en/products/detail/bourns-inc/CR1206-JW-512ELF/3925471</t>
-  </si>
-  <si>
-    <t>https://www.digikey.ca/en/products/detail/kingbright/WP154A4SUREQBFZGC/3084119</t>
-  </si>
-  <si>
-    <t>https://www.digikey.ca/en/products/detail/alps-alpine/SKRPABE010/18768948</t>
-  </si>
-  <si>
-    <t>https://www.digikey.ca/en/products/detail/littelfuse-inc./LR103G0J/3046801</t>
-  </si>
-  <si>
-    <t>Total:</t>
-  </si>
-  <si>
-    <t>YOCERA AVX</t>
-  </si>
-  <si>
-    <t>Kingbright</t>
-  </si>
-  <si>
-    <t>Littlefuse</t>
-  </si>
-  <si>
-    <t>Bourns</t>
-  </si>
-  <si>
-    <t>Würth Elektronik</t>
-  </si>
-  <si>
-    <t>Murata Electronics</t>
-  </si>
-  <si>
-    <t>Abracon LLC</t>
-  </si>
-  <si>
-    <t>Same Sky</t>
-  </si>
-  <si>
-    <t>Alpine</t>
+    <t>https://www.digikey.ca/en/products/detail/kemet/C0805C104K5RACTU/411169</t>
+  </si>
+  <si>
+    <t>0.1uF Ceramic Capacitor</t>
+  </si>
+  <si>
+    <t>https://www.digikey.ca/en/products/detail/stackpole-electronics-inc/RMCF0805FT10K0/1760676</t>
+  </si>
+  <si>
+    <t>Stackpole Electronics Inc</t>
+  </si>
+  <si>
+    <t>https://www.digikey.ca/en/products/detail/same-sky-formerly-cui-devices/CMC-5042PF-AC/1869984?s=N4IgTCBcDaIMIFk4FoCsAGALGACgMWQEE4QBdAXyA</t>
+  </si>
+  <si>
+    <t>Custom</t>
+  </si>
+  <si>
+    <t>Microphone</t>
+  </si>
+  <si>
+    <t>MK1</t>
+  </si>
+  <si>
+    <t>https://www.digikey.ca/en/products/detail/analog-devices-inc-maxim-integrated/MAX4466EXK-T/1781624</t>
+  </si>
+  <si>
+    <t>5-TSSOP, SC-70-5, SOT-353</t>
+  </si>
+  <si>
+    <t>Microphone Preamplifier</t>
+  </si>
+  <si>
+    <t>U3</t>
+  </si>
+  <si>
+    <t>R8, R9</t>
+  </si>
+  <si>
+    <t>2k Resistor</t>
+  </si>
+  <si>
+    <t>https://www.digikey.ca/en/products/detail/panasonic-electronic-components/ERA-6AEB202V/1465756</t>
+  </si>
+  <si>
+    <t>Panasonic Electronic Components</t>
+  </si>
+  <si>
+    <t>R10, R11</t>
+  </si>
+  <si>
+    <t>1M Resistor</t>
+  </si>
+  <si>
+    <t>R12, R13</t>
+  </si>
+  <si>
+    <t>https://www.digikey.ca/en/products/detail/panasonic-electronic-components/ERJ-3EKF1004V/196033</t>
+  </si>
+  <si>
+    <t>100k Resistor</t>
+  </si>
+  <si>
+    <t>https://www.digikey.ca/en/products/detail/panasonic-electronic-components/ERA-6AEB104V/1465797</t>
+  </si>
+  <si>
+    <t>R14</t>
+  </si>
+  <si>
+    <t>C6, C7, C8, C9</t>
   </si>
 </sst>
 </file>
@@ -242,7 +308,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="44" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="170" formatCode="&quot;$&quot;#,##0.00"/>
+    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -333,9 +399,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -345,10 +414,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -368,8 +433,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{4EBD2449-A99C-4B50-A989-B11F8DF9214D}" name="Table2" displayName="Table2" ref="A2:J14" totalsRowShown="0">
-  <autoFilter ref="A2:J14" xr:uid="{4EBD2449-A99C-4B50-A989-B11F8DF9214D}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{4EBD2449-A99C-4B50-A989-B11F8DF9214D}" name="Table2" displayName="Table2" ref="A2:J21" totalsRowShown="0">
+  <autoFilter ref="A2:J21" xr:uid="{4EBD2449-A99C-4B50-A989-B11F8DF9214D}"/>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{7FC96545-2991-43EA-8EEE-F1E652BE326F}" name="Item #"/>
     <tableColumn id="2" xr3:uid="{9FB5BFE9-D765-40F5-BF3E-56CCC6E7B618}" name="Designator"/>
@@ -705,34 +770,35 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B8654E07-79A6-40F1-9F87-AE3BAF6E2669}">
-  <dimension ref="A1:J16"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:J23"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="8.7109375" customWidth="1"/>
-    <col min="2" max="2" width="21.28515625" customWidth="1"/>
-    <col min="3" max="3" width="28.7109375" customWidth="1"/>
-    <col min="4" max="5" width="21" customWidth="1"/>
-    <col min="6" max="6" width="19" customWidth="1"/>
-    <col min="7" max="7" width="14.42578125" customWidth="1"/>
-    <col min="8" max="8" width="10.85546875" customWidth="1"/>
-    <col min="10" max="10" width="93.85546875" customWidth="1"/>
+    <col min="1" max="1" width="8.7265625" customWidth="1"/>
+    <col min="2" max="2" width="21.26953125" customWidth="1"/>
+    <col min="3" max="3" width="29" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="31.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21" customWidth="1"/>
+    <col min="6" max="6" width="27.36328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.453125" customWidth="1"/>
+    <col min="8" max="8" width="10.81640625" customWidth="1"/>
+    <col min="10" max="10" width="93.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:10" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
-      <c r="H1" s="3"/>
-      <c r="I1" s="3"/>
-      <c r="J1" s="4"/>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6"/>
+      <c r="H1" s="6"/>
+      <c r="I1" s="6"/>
+      <c r="J1" s="7"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -764,7 +830,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>1</v>
       </c>
@@ -783,7 +849,7 @@
       <c r="F3" t="s">
         <v>14</v>
       </c>
-      <c r="G3" s="5">
+      <c r="G3" s="2">
         <v>2.5099999999999998</v>
       </c>
       <c r="H3">
@@ -797,7 +863,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>2</v>
       </c>
@@ -805,32 +871,32 @@
         <v>17</v>
       </c>
       <c r="C4" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="D4" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="E4" t="s">
         <v>12</v>
       </c>
       <c r="F4" t="s">
-        <v>37</v>
-      </c>
-      <c r="G4" s="5">
+        <v>31</v>
+      </c>
+      <c r="G4" s="2">
         <v>0.26</v>
       </c>
       <c r="H4">
         <v>2</v>
       </c>
       <c r="I4" s="1">
-        <f t="shared" ref="I4:I14" si="0">G4*H4</f>
+        <f t="shared" ref="I4:I10" si="0">G4*H4</f>
         <v>0.52</v>
       </c>
       <c r="J4" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>3</v>
       </c>
@@ -838,18 +904,18 @@
         <v>18</v>
       </c>
       <c r="C5" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="D5" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="E5" t="s">
         <v>12</v>
       </c>
       <c r="F5" t="s">
-        <v>37</v>
-      </c>
-      <c r="G5" s="5">
+        <v>31</v>
+      </c>
+      <c r="G5" s="2">
         <v>0.35</v>
       </c>
       <c r="H5">
@@ -860,29 +926,29 @@
         <v>0.7</v>
       </c>
       <c r="J5" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="C6" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="D6" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="E6" t="s">
         <v>12</v>
       </c>
       <c r="F6" t="s">
-        <v>37</v>
-      </c>
-      <c r="G6" s="5">
+        <v>31</v>
+      </c>
+      <c r="G6" s="2">
         <v>0.45</v>
       </c>
       <c r="H6">
@@ -893,10 +959,10 @@
         <v>0.45</v>
       </c>
       <c r="J6" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>5</v>
       </c>
@@ -907,15 +973,15 @@
         <v>20</v>
       </c>
       <c r="D7" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="E7" t="s">
         <v>12</v>
       </c>
       <c r="F7" t="s">
-        <v>45</v>
-      </c>
-      <c r="G7" s="5">
+        <v>39</v>
+      </c>
+      <c r="G7" s="2">
         <v>1.05</v>
       </c>
       <c r="H7">
@@ -925,11 +991,11 @@
         <f t="shared" si="0"/>
         <v>1.05</v>
       </c>
-      <c r="J7" s="8" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J7" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>6</v>
       </c>
@@ -937,18 +1003,18 @@
         <v>21</v>
       </c>
       <c r="C8" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D8" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="E8" t="s">
         <v>12</v>
       </c>
       <c r="F8" t="s">
-        <v>42</v>
-      </c>
-      <c r="G8" s="5">
+        <v>36</v>
+      </c>
+      <c r="G8" s="2">
         <v>0.28999999999999998</v>
       </c>
       <c r="H8">
@@ -959,10 +1025,10 @@
         <v>0.57999999999999996</v>
       </c>
       <c r="J8" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>7</v>
       </c>
@@ -970,18 +1036,18 @@
         <v>22</v>
       </c>
       <c r="C9" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="D9" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="E9" t="s">
         <v>12</v>
       </c>
       <c r="F9" t="s">
-        <v>42</v>
-      </c>
-      <c r="G9" s="5">
+        <v>36</v>
+      </c>
+      <c r="G9" s="2">
         <v>0.18</v>
       </c>
       <c r="H9">
@@ -992,10 +1058,10 @@
         <v>0.54</v>
       </c>
       <c r="J9" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>8</v>
       </c>
@@ -1003,18 +1069,18 @@
         <v>23</v>
       </c>
       <c r="C10" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="D10" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="E10" t="s">
         <v>12</v>
       </c>
       <c r="F10" t="s">
-        <v>42</v>
-      </c>
-      <c r="G10" s="5">
+        <v>36</v>
+      </c>
+      <c r="G10" s="2">
         <v>0.15</v>
       </c>
       <c r="H10">
@@ -1025,10 +1091,10 @@
         <v>0.3</v>
       </c>
       <c r="J10" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>9</v>
       </c>
@@ -1036,32 +1102,29 @@
         <v>24</v>
       </c>
       <c r="C11" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="D11" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="E11" t="s">
         <v>12</v>
       </c>
-      <c r="F11" t="s">
-        <v>42</v>
-      </c>
-      <c r="G11" s="5">
-        <v>1.4</v>
+      <c r="G11" s="2">
+        <v>0.59</v>
       </c>
       <c r="H11">
         <v>1</v>
       </c>
       <c r="I11" s="1">
-        <f t="shared" si="0"/>
-        <v>1.4</v>
+        <f t="shared" ref="I11:I20" si="1">G11*H11</f>
+        <v>0.59</v>
       </c>
       <c r="J11" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>10</v>
       </c>
@@ -1069,99 +1132,327 @@
         <v>25</v>
       </c>
       <c r="C12" t="s">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="D12" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="E12" t="s">
-        <v>35</v>
-      </c>
-      <c r="F12" t="s">
-        <v>36</v>
-      </c>
-      <c r="G12" s="5">
-        <v>0.99</v>
+        <v>12</v>
+      </c>
+      <c r="G12" s="2">
+        <v>0.32</v>
       </c>
       <c r="H12">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="I12" s="1">
-        <f t="shared" si="0"/>
-        <v>0.99</v>
+        <f t="shared" si="1"/>
+        <v>3.2</v>
       </c>
       <c r="J12" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>26</v>
+        <v>58</v>
       </c>
       <c r="C13" t="s">
-        <v>28</v>
+        <v>57</v>
       </c>
       <c r="D13" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="E13" t="s">
         <v>12</v>
       </c>
-      <c r="G13" s="5">
-        <v>0.59</v>
+      <c r="F13" t="s">
+        <v>59</v>
+      </c>
+      <c r="G13" s="2">
+        <v>27.91</v>
       </c>
       <c r="H13">
         <v>1</v>
       </c>
       <c r="I13" s="1">
-        <f t="shared" si="0"/>
-        <v>0.59</v>
+        <f t="shared" si="1"/>
+        <v>27.91</v>
       </c>
       <c r="J13" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>12</v>
       </c>
       <c r="B14" t="s">
+        <v>87</v>
+      </c>
+      <c r="C14" t="s">
+        <v>65</v>
+      </c>
+      <c r="D14" t="s">
+        <v>32</v>
+      </c>
+      <c r="E14" t="s">
+        <v>12</v>
+      </c>
+      <c r="F14" t="s">
+        <v>31</v>
+      </c>
+      <c r="G14" s="2">
+        <v>0.12</v>
+      </c>
+      <c r="H14">
+        <v>10</v>
+      </c>
+      <c r="I14" s="1">
+        <f t="shared" si="1"/>
+        <v>1.2</v>
+      </c>
+      <c r="J14" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A15">
+        <v>13</v>
+      </c>
+      <c r="B15" t="s">
+        <v>76</v>
+      </c>
+      <c r="C15" t="s">
         <v>27</v>
       </c>
-      <c r="C14" t="s">
-        <v>44</v>
-      </c>
-      <c r="D14" t="s">
-        <v>65</v>
-      </c>
-      <c r="E14" t="s">
-        <v>12</v>
-      </c>
-      <c r="G14" s="5">
-        <v>0.32</v>
-      </c>
-      <c r="H14">
+      <c r="D15" t="s">
+        <v>67</v>
+      </c>
+      <c r="E15" t="s">
+        <v>12</v>
+      </c>
+      <c r="F15" t="s">
+        <v>31</v>
+      </c>
+      <c r="G15" s="2">
+        <v>0.15</v>
+      </c>
+      <c r="H15">
+        <v>10</v>
+      </c>
+      <c r="I15" s="1">
+        <f t="shared" si="1"/>
+        <v>1.5</v>
+      </c>
+      <c r="J15" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A16">
+        <v>14</v>
+      </c>
+      <c r="B16" t="s">
+        <v>71</v>
+      </c>
+      <c r="C16" t="s">
+        <v>70</v>
+      </c>
+      <c r="D16" t="s">
+        <v>54</v>
+      </c>
+      <c r="E16" t="s">
+        <v>63</v>
+      </c>
+      <c r="G16" s="2">
+        <v>1.89</v>
+      </c>
+      <c r="H16">
+        <v>3</v>
+      </c>
+      <c r="I16" s="1">
+        <f t="shared" si="1"/>
+        <v>5.67</v>
+      </c>
+      <c r="J16" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A17">
+        <v>15</v>
+      </c>
+      <c r="B17" t="s">
+        <v>75</v>
+      </c>
+      <c r="C17" t="s">
+        <v>74</v>
+      </c>
+      <c r="D17" t="s">
+        <v>56</v>
+      </c>
+      <c r="E17" t="s">
+        <v>12</v>
+      </c>
+      <c r="F17" t="s">
+        <v>73</v>
+      </c>
+      <c r="G17" s="2">
+        <v>1.51</v>
+      </c>
+      <c r="H17">
+        <v>3</v>
+      </c>
+      <c r="I17" s="1">
+        <f t="shared" si="1"/>
+        <v>4.53</v>
+      </c>
+      <c r="J17" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A18">
+        <v>16</v>
+      </c>
+      <c r="B18" t="s">
+        <v>80</v>
+      </c>
+      <c r="C18" t="s">
+        <v>77</v>
+      </c>
+      <c r="D18" t="s">
+        <v>79</v>
+      </c>
+      <c r="E18" t="s">
+        <v>12</v>
+      </c>
+      <c r="F18" t="s">
+        <v>31</v>
+      </c>
+      <c r="G18" s="2">
+        <v>0.15</v>
+      </c>
+      <c r="H18">
+        <v>5</v>
+      </c>
+      <c r="I18" s="1">
+        <f t="shared" si="1"/>
+        <v>0.75</v>
+      </c>
+      <c r="J18" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A19">
+        <v>17</v>
+      </c>
+      <c r="B19" t="s">
+        <v>82</v>
+      </c>
+      <c r="C19" t="s">
+        <v>81</v>
+      </c>
+      <c r="D19" t="s">
+        <v>79</v>
+      </c>
+      <c r="E19" t="s">
+        <v>12</v>
+      </c>
+      <c r="F19" t="s">
+        <v>31</v>
+      </c>
+      <c r="G19" s="2">
+        <v>0.15</v>
+      </c>
+      <c r="H19">
+        <v>5</v>
+      </c>
+      <c r="I19" s="1">
+        <f t="shared" si="1"/>
+        <v>0.75</v>
+      </c>
+      <c r="J19" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A20">
+        <v>18</v>
+      </c>
+      <c r="B20" t="s">
+        <v>86</v>
+      </c>
+      <c r="C20" t="s">
+        <v>84</v>
+      </c>
+      <c r="D20" t="s">
+        <v>79</v>
+      </c>
+      <c r="E20" t="s">
+        <v>12</v>
+      </c>
+      <c r="F20" t="s">
+        <v>31</v>
+      </c>
+      <c r="G20" s="2">
+        <v>0.15</v>
+      </c>
+      <c r="H20">
+        <v>5</v>
+      </c>
+      <c r="I20" s="1">
+        <f t="shared" si="1"/>
+        <v>0.75</v>
+      </c>
+      <c r="J20" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A21">
+        <v>21</v>
+      </c>
+      <c r="C21" t="s">
+        <v>62</v>
+      </c>
+      <c r="D21" t="s">
+        <v>61</v>
+      </c>
+      <c r="E21" t="s">
+        <v>63</v>
+      </c>
+      <c r="F21" t="s">
+        <v>69</v>
+      </c>
+      <c r="G21" s="2">
+        <v>0</v>
+      </c>
+      <c r="H21">
         <v>1</v>
       </c>
-      <c r="I14" s="1">
-        <f t="shared" si="0"/>
-        <v>0.32</v>
-      </c>
-      <c r="J14" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="16" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="H16" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="I16" s="7">
+      <c r="I21" s="1">
+        <f t="shared" ref="I21" si="2">G21*H21</f>
+        <v>0</v>
+      </c>
+      <c r="J21" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="23" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="H23" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="I23" s="4">
         <f>SUM(Table2[Total])</f>
-        <v>9.9499999999999993</v>
+        <v>53.500000000000007</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
finished schematic. updated BOM. stuff.
</commit_message>
<xml_diff>
--- a/RESOURCES/BOM/BOM.xlsx
+++ b/RESOURCES/BOM/BOM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nicoj\Documents\Repositories\MIST\RESOURCES\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3385EE7-1C50-47BB-936D-302565A7D705}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3373818B-4870-4F70-985C-34221BD32FBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2280" yWindow="2280" windowWidth="19200" windowHeight="11170" xr2:uid="{26158271-47B5-455E-A3AA-B8B46F5ACF1D}"/>
+    <workbookView xWindow="3190" yWindow="2080" windowWidth="19200" windowHeight="11180" xr2:uid="{26158271-47B5-455E-A3AA-B8B46F5ACF1D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="81">
   <si>
     <t xml:space="preserve">Bill Of Material - Project Template </t>
   </si>
@@ -68,9 +68,6 @@
     <t>U1</t>
   </si>
   <si>
-    <t>AtMega328PU</t>
-  </si>
-  <si>
     <t>Atmel</t>
   </si>
   <si>
@@ -101,30 +98,18 @@
     <t>16Mhz Crystal Osillator</t>
   </si>
   <si>
-    <t>R1, R2</t>
-  </si>
-  <si>
-    <t>R3, R4, R5</t>
-  </si>
-  <si>
     <t>R6, R7</t>
   </si>
   <si>
     <t>J2</t>
   </si>
   <si>
-    <t>S1</t>
-  </si>
-  <si>
     <t>USB Type C Power Only</t>
   </si>
   <si>
     <t>10k Resistor</t>
   </si>
   <si>
-    <t>220 Resistor</t>
-  </si>
-  <si>
     <t>5.1K Resistor</t>
   </si>
   <si>
@@ -170,12 +155,6 @@
     <t>https://www.digikey.ca/en/products/detail/kemet/C0805C104J5RACAUTO/3314435</t>
   </si>
   <si>
-    <t>https://www.digikey.ca/en/products/detail/w-rth-elektronik/560112132015/24849722</t>
-  </si>
-  <si>
-    <t>https://www.digikey.ca/en/products/detail/bourns-inc/CRM1206AJW-103ELF/8258196</t>
-  </si>
-  <si>
     <t>https://www.digikey.ca/en/products/detail/bourns-inc/CR1206-JW-512ELF/3925471</t>
   </si>
   <si>
@@ -188,12 +167,6 @@
     <t>Littlefuse</t>
   </si>
   <si>
-    <t>Bourns</t>
-  </si>
-  <si>
-    <t>Würth Elektronik</t>
-  </si>
-  <si>
     <t>Murata Electronics</t>
   </si>
   <si>
@@ -278,15 +251,9 @@
     <t>Panasonic Electronic Components</t>
   </si>
   <si>
-    <t>R10, R11</t>
-  </si>
-  <si>
     <t>1M Resistor</t>
   </si>
   <si>
-    <t>R12, R13</t>
-  </si>
-  <si>
     <t>https://www.digikey.ca/en/products/detail/panasonic-electronic-components/ERJ-3EKF1004V/196033</t>
   </si>
   <si>
@@ -296,10 +263,22 @@
     <t>https://www.digikey.ca/en/products/detail/panasonic-electronic-components/ERA-6AEB104V/1465797</t>
   </si>
   <si>
-    <t>R14</t>
-  </si>
-  <si>
     <t>C6, C7, C8, C9</t>
+  </si>
+  <si>
+    <t>R4, R5</t>
+  </si>
+  <si>
+    <t>R10</t>
+  </si>
+  <si>
+    <t>R1, R2, R3</t>
+  </si>
+  <si>
+    <t>AtMega328PB</t>
+  </si>
+  <si>
+    <t>S1, S2</t>
   </si>
 </sst>
 </file>
@@ -433,8 +412,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{4EBD2449-A99C-4B50-A989-B11F8DF9214D}" name="Table2" displayName="Table2" ref="A2:J21" totalsRowShown="0">
-  <autoFilter ref="A2:J21" xr:uid="{4EBD2449-A99C-4B50-A989-B11F8DF9214D}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{4EBD2449-A99C-4B50-A989-B11F8DF9214D}" name="Table2" displayName="Table2" ref="A2:J19" totalsRowShown="0">
+  <autoFilter ref="A2:J19" xr:uid="{4EBD2449-A99C-4B50-A989-B11F8DF9214D}"/>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{7FC96545-2991-43EA-8EEE-F1E652BE326F}" name="Item #"/>
     <tableColumn id="2" xr3:uid="{9FB5BFE9-D765-40F5-BF3E-56CCC6E7B618}" name="Designator"/>
@@ -770,7 +749,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B8654E07-79A6-40F1-9F87-AE3BAF6E2669}">
-  <dimension ref="A1:J23"/>
+  <dimension ref="A1:J21"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="8.7265625" customWidth="1"/>
@@ -806,7 +785,7 @@
         <v>2</v>
       </c>
       <c r="C2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D2" t="s">
         <v>3</v>
@@ -815,7 +794,7 @@
         <v>4</v>
       </c>
       <c r="F2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G2" t="s">
         <v>5</v>
@@ -838,16 +817,16 @@
         <v>9</v>
       </c>
       <c r="C3" t="s">
+        <v>79</v>
+      </c>
+      <c r="D3" t="s">
         <v>10</v>
       </c>
-      <c r="D3" t="s">
-        <v>11</v>
-      </c>
       <c r="E3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G3" s="2">
         <v>2.5099999999999998</v>
@@ -860,7 +839,7 @@
         <v>2.5099999999999998</v>
       </c>
       <c r="J3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.35">
@@ -868,19 +847,19 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C4" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="D4" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="E4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F4" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="G4" s="2">
         <v>0.26</v>
@@ -889,11 +868,11 @@
         <v>2</v>
       </c>
       <c r="I4" s="1">
-        <f t="shared" ref="I4:I10" si="0">G4*H4</f>
+        <f t="shared" ref="I4:I9" si="0">G4*H4</f>
         <v>0.52</v>
       </c>
       <c r="J4" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.35">
@@ -901,19 +880,19 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C5" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="D5" t="s">
-        <v>52</v>
+        <v>43</v>
       </c>
       <c r="E5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F5" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="G5" s="2">
         <v>0.35</v>
@@ -926,7 +905,7 @@
         <v>0.7</v>
       </c>
       <c r="J5" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.35">
@@ -934,19 +913,19 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" t="s">
         <v>30</v>
       </c>
-      <c r="C6" t="s">
-        <v>35</v>
-      </c>
       <c r="D6" t="s">
-        <v>52</v>
+        <v>43</v>
       </c>
       <c r="E6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F6" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="G6" s="2">
         <v>0.45</v>
@@ -959,7 +938,7 @@
         <v>0.45</v>
       </c>
       <c r="J6" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.35">
@@ -967,19 +946,19 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" t="s">
         <v>19</v>
       </c>
-      <c r="C7" t="s">
-        <v>20</v>
-      </c>
       <c r="D7" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="E7" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F7" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="G7" s="2">
         <v>1.05</v>
@@ -992,7 +971,7 @@
         <v>1.05</v>
       </c>
       <c r="J7" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.35">
@@ -1000,32 +979,32 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>21</v>
+        <v>78</v>
       </c>
       <c r="C8" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="D8" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="E8" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F8" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="G8" s="2">
-        <v>0.28999999999999998</v>
+        <v>0.15</v>
       </c>
       <c r="H8">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="I8" s="1">
         <f t="shared" si="0"/>
-        <v>0.57999999999999996</v>
+        <v>1.5</v>
       </c>
       <c r="J8" t="s">
-        <v>45</v>
+        <v>57</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.35">
@@ -1033,32 +1012,32 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>22</v>
+        <v>76</v>
       </c>
       <c r="C9" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D9" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="E9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F9" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="G9" s="2">
-        <v>0.18</v>
+        <v>0.15</v>
       </c>
       <c r="H9">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I9" s="1">
         <f t="shared" si="0"/>
-        <v>0.54</v>
+        <v>0.3</v>
       </c>
       <c r="J9" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.35">
@@ -1066,32 +1045,29 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C10" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="D10" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="E10" t="s">
-        <v>12</v>
-      </c>
-      <c r="F10" t="s">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="G10" s="2">
-        <v>0.15</v>
+        <v>0.59</v>
       </c>
       <c r="H10">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I10" s="1">
-        <f t="shared" si="0"/>
-        <v>0.3</v>
+        <f t="shared" ref="I10:I18" si="1">G10*H10</f>
+        <v>0.59</v>
       </c>
       <c r="J10" t="s">
-        <v>46</v>
+        <v>32</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.35">
@@ -1099,29 +1075,29 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>24</v>
+        <v>80</v>
       </c>
       <c r="C11" t="s">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="D11" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="E11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G11" s="2">
-        <v>0.59</v>
+        <v>0.32</v>
       </c>
       <c r="H11">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="I11" s="1">
-        <f t="shared" ref="I11:I20" si="1">G11*H11</f>
-        <v>0.59</v>
+        <f t="shared" si="1"/>
+        <v>3.2</v>
       </c>
       <c r="J11" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.35">
@@ -1129,29 +1105,32 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="C12" t="s">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="D12" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E12" t="s">
-        <v>12</v>
+        <v>11</v>
+      </c>
+      <c r="F12" t="s">
+        <v>50</v>
       </c>
       <c r="G12" s="2">
-        <v>0.32</v>
+        <v>27.91</v>
       </c>
       <c r="H12">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="I12" s="1">
         <f t="shared" si="1"/>
-        <v>3.2</v>
+        <v>27.91</v>
       </c>
       <c r="J12" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.35">
@@ -1159,32 +1138,32 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="C13" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D13" t="s">
-        <v>56</v>
+        <v>27</v>
       </c>
       <c r="E13" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F13" t="s">
-        <v>59</v>
+        <v>26</v>
       </c>
       <c r="G13" s="2">
-        <v>27.91</v>
+        <v>0.12</v>
       </c>
       <c r="H13">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="I13" s="1">
         <f t="shared" si="1"/>
-        <v>27.91</v>
+        <v>1.2</v>
       </c>
       <c r="J13" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.35">
@@ -1192,32 +1171,29 @@
         <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>87</v>
+        <v>62</v>
       </c>
       <c r="C14" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="D14" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="E14" t="s">
-        <v>12</v>
-      </c>
-      <c r="F14" t="s">
-        <v>31</v>
+        <v>54</v>
       </c>
       <c r="G14" s="2">
-        <v>0.12</v>
+        <v>1.89</v>
       </c>
       <c r="H14">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="I14" s="1">
         <f t="shared" si="1"/>
-        <v>1.2</v>
+        <v>5.67</v>
       </c>
       <c r="J14" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.35">
@@ -1225,32 +1201,32 @@
         <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="C15" t="s">
-        <v>27</v>
+        <v>65</v>
       </c>
       <c r="D15" t="s">
-        <v>67</v>
+        <v>47</v>
       </c>
       <c r="E15" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F15" t="s">
-        <v>31</v>
+        <v>64</v>
       </c>
       <c r="G15" s="2">
-        <v>0.15</v>
+        <v>1.51</v>
       </c>
       <c r="H15">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="I15" s="1">
         <f t="shared" si="1"/>
-        <v>1.5</v>
+        <v>4.53</v>
       </c>
       <c r="J15" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.35">
@@ -1258,29 +1234,32 @@
         <v>14</v>
       </c>
       <c r="B16" t="s">
-        <v>71</v>
+        <v>20</v>
       </c>
       <c r="C16" t="s">
+        <v>68</v>
+      </c>
+      <c r="D16" t="s">
         <v>70</v>
       </c>
-      <c r="D16" t="s">
-        <v>54</v>
-      </c>
       <c r="E16" t="s">
-        <v>63</v>
+        <v>11</v>
+      </c>
+      <c r="F16" t="s">
+        <v>26</v>
       </c>
       <c r="G16" s="2">
-        <v>1.89</v>
+        <v>0.15</v>
       </c>
       <c r="H16">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I16" s="1">
         <f t="shared" si="1"/>
-        <v>5.67</v>
+        <v>0.75</v>
       </c>
       <c r="J16" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.35">
@@ -1288,29 +1267,29 @@
         <v>15</v>
       </c>
       <c r="B17" t="s">
-        <v>75</v>
+        <v>67</v>
       </c>
       <c r="C17" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="D17" t="s">
-        <v>56</v>
+        <v>70</v>
       </c>
       <c r="E17" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F17" t="s">
-        <v>73</v>
+        <v>26</v>
       </c>
       <c r="G17" s="2">
-        <v>1.51</v>
+        <v>0.15</v>
       </c>
       <c r="H17">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I17" s="1">
         <f t="shared" si="1"/>
-        <v>4.53</v>
+        <v>0.75</v>
       </c>
       <c r="J17" t="s">
         <v>72</v>
@@ -1321,19 +1300,19 @@
         <v>16</v>
       </c>
       <c r="B18" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="C18" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="D18" t="s">
-        <v>79</v>
+        <v>70</v>
       </c>
       <c r="E18" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F18" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="G18" s="2">
         <v>0.15</v>
@@ -1346,113 +1325,47 @@
         <v>0.75</v>
       </c>
       <c r="J18" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>17</v>
       </c>
-      <c r="B19" t="s">
-        <v>82</v>
-      </c>
       <c r="C19" t="s">
-        <v>81</v>
+        <v>53</v>
       </c>
       <c r="D19" t="s">
-        <v>79</v>
+        <v>52</v>
       </c>
       <c r="E19" t="s">
-        <v>12</v>
+        <v>54</v>
       </c>
       <c r="F19" t="s">
-        <v>31</v>
+        <v>60</v>
       </c>
       <c r="G19" s="2">
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="H19">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I19" s="1">
-        <f t="shared" si="1"/>
-        <v>0.75</v>
+        <f t="shared" ref="I19" si="2">G19*H19</f>
+        <v>0</v>
       </c>
       <c r="J19" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A20">
-        <v>18</v>
-      </c>
-      <c r="B20" t="s">
-        <v>86</v>
-      </c>
-      <c r="C20" t="s">
-        <v>84</v>
-      </c>
-      <c r="D20" t="s">
-        <v>79</v>
-      </c>
-      <c r="E20" t="s">
-        <v>12</v>
-      </c>
-      <c r="F20" t="s">
-        <v>31</v>
-      </c>
-      <c r="G20" s="2">
-        <v>0.15</v>
-      </c>
-      <c r="H20">
-        <v>5</v>
-      </c>
-      <c r="I20" s="1">
-        <f t="shared" si="1"/>
-        <v>0.75</v>
-      </c>
-      <c r="J20" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A21">
-        <v>21</v>
-      </c>
-      <c r="C21" t="s">
-        <v>62</v>
-      </c>
-      <c r="D21" t="s">
-        <v>61</v>
-      </c>
-      <c r="E21" t="s">
-        <v>63</v>
-      </c>
-      <c r="F21" t="s">
-        <v>69</v>
-      </c>
-      <c r="G21" s="2">
-        <v>0</v>
-      </c>
-      <c r="H21">
-        <v>1</v>
-      </c>
-      <c r="I21" s="1">
-        <f t="shared" ref="I21" si="2">G21*H21</f>
-        <v>0</v>
-      </c>
-      <c r="J21" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="23" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="H23" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="I23" s="4">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="21" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="H21" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="I21" s="4">
         <f>SUM(Table2[Total])</f>
-        <v>53.500000000000007</v>
+        <v>52.38000000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
finished schematic and layout
</commit_message>
<xml_diff>
--- a/RESOURCES/BOM/BOM.xlsx
+++ b/RESOURCES/BOM/BOM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nicoj\Documents\Repositories\MIST\RESOURCES\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3373818B-4870-4F70-985C-34221BD32FBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76DC70EC-A64A-42A5-9479-A59C44575528}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3190" yWindow="2080" windowWidth="19200" windowHeight="11180" xr2:uid="{26158271-47B5-455E-A3AA-B8B46F5ACF1D}"/>
+    <workbookView xWindow="1630" yWindow="3160" windowWidth="19200" windowHeight="11180" xr2:uid="{26158271-47B5-455E-A3AA-B8B46F5ACF1D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="79">
   <si>
     <t xml:space="preserve">Bill Of Material - Project Template </t>
   </si>
@@ -131,9 +131,6 @@
     <t>22uF Ceramic Capacitor</t>
   </si>
   <si>
-    <t>1206 (3216 Metric)</t>
-  </si>
-  <si>
     <t>https://www.digikey.ca/en/products/detail/same-sky-formerly-cui-devices/UJC-H-G-SMT-P6-TR/24818614</t>
   </si>
   <si>
@@ -155,18 +152,12 @@
     <t>https://www.digikey.ca/en/products/detail/kemet/C0805C104J5RACAUTO/3314435</t>
   </si>
   <si>
-    <t>https://www.digikey.ca/en/products/detail/bourns-inc/CR1206-JW-512ELF/3925471</t>
-  </si>
-  <si>
     <t>https://www.digikey.ca/en/products/detail/alps-alpine/SKRPABE010/18768948</t>
   </si>
   <si>
     <t>Total:</t>
   </si>
   <si>
-    <t>Littlefuse</t>
-  </si>
-  <si>
     <t>Murata Electronics</t>
   </si>
   <si>
@@ -279,6 +270,9 @@
   </si>
   <si>
     <t>S1, S2</t>
+  </si>
+  <si>
+    <t>https://www.digikey.ca/en/products/detail/stackpole-electronics-inc/RMCF0805JT5K10/1757930</t>
   </si>
 </sst>
 </file>
@@ -817,7 +811,7 @@
         <v>9</v>
       </c>
       <c r="C3" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="D3" t="s">
         <v>10</v>
@@ -872,7 +866,7 @@
         <v>0.52</v>
       </c>
       <c r="J4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.35">
@@ -886,7 +880,7 @@
         <v>29</v>
       </c>
       <c r="D5" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="E5" t="s">
         <v>11</v>
@@ -905,7 +899,7 @@
         <v>0.7</v>
       </c>
       <c r="J5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.35">
@@ -919,7 +913,7 @@
         <v>30</v>
       </c>
       <c r="D6" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="E6" t="s">
         <v>11</v>
@@ -938,7 +932,7 @@
         <v>0.45</v>
       </c>
       <c r="J6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.35">
@@ -952,13 +946,13 @@
         <v>19</v>
       </c>
       <c r="D7" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="E7" t="s">
         <v>11</v>
       </c>
       <c r="F7" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G7" s="2">
         <v>1.05</v>
@@ -971,7 +965,7 @@
         <v>1.05</v>
       </c>
       <c r="J7" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.35">
@@ -979,13 +973,13 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="C8" t="s">
         <v>23</v>
       </c>
       <c r="D8" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="E8" t="s">
         <v>11</v>
@@ -1004,7 +998,7 @@
         <v>1.5</v>
       </c>
       <c r="J8" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.35">
@@ -1012,32 +1006,32 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C9" t="s">
         <v>24</v>
       </c>
       <c r="D9" t="s">
-        <v>42</v>
+        <v>55</v>
       </c>
       <c r="E9" t="s">
         <v>11</v>
       </c>
       <c r="F9" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="G9" s="2">
-        <v>0.15</v>
+        <v>0.16</v>
       </c>
       <c r="H9">
         <v>2</v>
       </c>
       <c r="I9" s="1">
         <f t="shared" si="0"/>
-        <v>0.3</v>
+        <v>0.32</v>
       </c>
       <c r="J9" t="s">
-        <v>39</v>
+        <v>78</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.35">
@@ -1051,7 +1045,7 @@
         <v>22</v>
       </c>
       <c r="D10" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="E10" t="s">
         <v>11</v>
@@ -1067,7 +1061,7 @@
         <v>0.59</v>
       </c>
       <c r="J10" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.35">
@@ -1075,13 +1069,13 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="C11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D11" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="E11" t="s">
         <v>11</v>
@@ -1097,7 +1091,7 @@
         <v>3.2</v>
       </c>
       <c r="J11" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.35">
@@ -1105,19 +1099,19 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="C12" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D12" t="s">
+        <v>44</v>
+      </c>
+      <c r="E12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F12" t="s">
         <v>47</v>
-      </c>
-      <c r="E12" t="s">
-        <v>11</v>
-      </c>
-      <c r="F12" t="s">
-        <v>50</v>
       </c>
       <c r="G12" s="2">
         <v>27.91</v>
@@ -1130,7 +1124,7 @@
         <v>27.91</v>
       </c>
       <c r="J12" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.35">
@@ -1138,10 +1132,10 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="C13" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="D13" t="s">
         <v>27</v>
@@ -1163,7 +1157,7 @@
         <v>1.2</v>
       </c>
       <c r="J13" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.35">
@@ -1171,16 +1165,16 @@
         <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C14" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="D14" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="E14" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="G14" s="2">
         <v>1.89</v>
@@ -1193,7 +1187,7 @@
         <v>5.67</v>
       </c>
       <c r="J14" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.35">
@@ -1201,19 +1195,19 @@
         <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="C15" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="D15" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="E15" t="s">
         <v>11</v>
       </c>
       <c r="F15" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="G15" s="2">
         <v>1.51</v>
@@ -1226,7 +1220,7 @@
         <v>4.53</v>
       </c>
       <c r="J15" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.35">
@@ -1237,10 +1231,10 @@
         <v>20</v>
       </c>
       <c r="C16" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="D16" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="E16" t="s">
         <v>11</v>
@@ -1259,7 +1253,7 @@
         <v>0.75</v>
       </c>
       <c r="J16" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.35">
@@ -1267,13 +1261,13 @@
         <v>15</v>
       </c>
       <c r="B17" t="s">
+        <v>64</v>
+      </c>
+      <c r="C17" t="s">
+        <v>68</v>
+      </c>
+      <c r="D17" t="s">
         <v>67</v>
-      </c>
-      <c r="C17" t="s">
-        <v>71</v>
-      </c>
-      <c r="D17" t="s">
-        <v>70</v>
       </c>
       <c r="E17" t="s">
         <v>11</v>
@@ -1292,7 +1286,7 @@
         <v>0.75</v>
       </c>
       <c r="J17" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.35">
@@ -1300,13 +1294,13 @@
         <v>16</v>
       </c>
       <c r="B18" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="C18" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="D18" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="E18" t="s">
         <v>11</v>
@@ -1325,7 +1319,7 @@
         <v>0.75</v>
       </c>
       <c r="J18" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.35">
@@ -1333,16 +1327,16 @@
         <v>17</v>
       </c>
       <c r="C19" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="D19" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="E19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F19" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="G19" s="2">
         <v>0</v>
@@ -1355,17 +1349,17 @@
         <v>0</v>
       </c>
       <c r="J19" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="21" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="H21" s="3" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="I21" s="4">
         <f>SUM(Table2[Total])</f>
-        <v>52.38000000000001</v>
+        <v>52.400000000000006</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fixed wrong matrix pin mappings schematic.
</commit_message>
<xml_diff>
--- a/RESOURCES/BOM/BOM.xlsx
+++ b/RESOURCES/BOM/BOM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nicoj\Documents\Repositories\MIST\RESOURCES\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76DC70EC-A64A-42A5-9479-A59C44575528}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D3CD23B-9A75-4717-9CFD-AAE9F4E49D7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1630" yWindow="3160" windowWidth="19200" windowHeight="11180" xr2:uid="{26158271-47B5-455E-A3AA-B8B46F5ACF1D}"/>
+    <workbookView xWindow="3190" yWindow="1980" windowWidth="19200" windowHeight="11170" xr2:uid="{26158271-47B5-455E-A3AA-B8B46F5ACF1D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>